<commit_message>
Corte 21-sep: la T01 sin entregar queda como NP
</commit_message>
<xml_diff>
--- a/calificaciones/P00-T01-corte-21sep.xlsx
+++ b/calificaciones/P00-T01-corte-21sep.xlsx
@@ -82,10 +82,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -459,13 +458,13 @@
   <dimension ref="A1:G44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="13" customWidth="1" style="2" min="1" max="1"/>
-    <col width="6" customWidth="1" style="2" min="2" max="2"/>
-    <col width="6" customWidth="1" style="2" min="3" max="3"/>
-    <col width="6" customWidth="1" style="2" min="4" max="4"/>
-    <col width="6" customWidth="1" style="2" min="5" max="5"/>
-    <col width="6" customWidth="1" style="2" min="6" max="6"/>
-    <col width="110" customWidth="1" style="2" min="7" max="7"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="6" customWidth="1" min="3" max="3"/>
+    <col width="6" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="6" customWidth="1" min="6" max="6"/>
+    <col width="110" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -485,50 +484,49 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>10 = correcta  ·  9 = correcta con un detalle  ·  8 = incompleta pero aceptada  ·  PC = pendiente de correccion (tienes hoja aparte)  ·  NP = no presentada  ·  — = aun no la subes y todavia no vence</t>
+          <t>10 = correcta  ·  9 = correcta con un detalle  ·  8 = incompleta pero aceptada  ·  PC = pendiente de correccion  ·  NP = no entregada al corte</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>P00: el objetivo era demostrar que sabes hacer push, asi que cuenta 10 para todo el que subio algo. T01: vencio el 14-sep; lo entregado hasta el 15-sep cuenta en tiempo por la prorroga que se dio en clase. PC = pendiente de correccion: no es una calificacion final, se recalifica en cuanto subas el arreglo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5"/>
+          <t>P00: el objetivo era demostrar que sabes hacer push, asi que cuenta 10 para todo el que subio algo. T01: vencio el lunes 14-sep, con la prorroga hasta el final de ese dia que se dio en clase; lo entregado el 15 tambien se conto. NP = no entregada al corte. Si la subes, avisame y la califico: la politica de entregas tardias de MPOO sigue sin definirse.</t>
+        </is>
+      </c>
+    </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Cuenta</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>P00</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>P01</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>P02</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>P03</t>
         </is>
       </c>
-      <c r="F6" s="3" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>T01</t>
         </is>
       </c>
-      <c r="G6" s="3" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>Observaciones</t>
         </is>
@@ -560,10 +558,10 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G7" s="4" t="inlineStr">
+          <t>NP</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
         <is>
           <t>P03 lista: tabla completa y analisis en el PDF (documento conjunto con otros dos companeros). En mis-resultados.txt dejaste en blanco los 'por que me equivoque', pero estan explicados en el PDF. Falta la T01.</t>
         </is>
@@ -600,7 +598,7 @@
           <t>PC</t>
         </is>
       </c>
-      <c r="G8" s="4" t="inlineStr">
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>Tu T01 quedo sin los .class: los borraste el 21-sep. El codigo compila bien con JDK 21 y el modelado y el quiz estan muy completos; recompila los tres y subelos para cerrarla.</t>
         </is>
@@ -637,7 +635,7 @@
           <t>10</t>
         </is>
       </c>
-      <c r="G9" s="4" t="inlineStr">
+      <c r="G9" s="3" t="inlineStr">
         <is>
           <t>Bloque 7 completo y buen analisis; tu captura no muestra la tabla final, solo el final del reporte. Tu T01 esta muy bien: 10. Dos detalles para la proxima: a Television le falto la linea QUE IGNORE, y entre las tres clases no usaste la resta.</t>
         </is>
@@ -671,10 +669,10 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G10" s="4" t="inlineStr">
+          <t>NP</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
         <is>
           <t>Faltan la P02 y la P03.</t>
         </is>
@@ -709,7 +707,7 @@
           <t>PC</t>
         </is>
       </c>
-      <c r="G11" s="4" t="inlineStr">
+      <c r="G11" s="3" t="inlineStr">
         <is>
           <t>P03 lista: tabla de 41 filas con analisis en PDF y captura. En la T01 faltan los tres .class y ningun metodo trae su '// firma:' en comentario.</t>
         </is>
@@ -744,7 +742,7 @@
       <c r="F12" t="n">
         <v>10</v>
       </c>
-      <c r="G12" s="4" t="inlineStr">
+      <c r="G12" s="3" t="inlineStr">
         <is>
           <t>T01 completa: los tres .class corren, el modelado tiene contexto propio y el quiz esta con tus palabras.</t>
         </is>
@@ -778,10 +776,10 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G13" s="4" t="inlineStr">
+          <t>NP</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
         <is>
           <t>Sin entregas registradas.</t>
         </is>
@@ -818,7 +816,7 @@
           <t>9</t>
         </is>
       </c>
-      <c r="G14" s="4" t="inlineStr">
+      <c r="G14" s="3" t="inlineStr">
         <is>
           <t>Completa. Detalle: tu explicacion del desbordamiento de Integer.MAX_VALUE quedo confusa. T01: 9. Te falto el operador %, MiCuaderno no tiene un metodo void con parametro y en el QUIZ la pregunta 1 no trae ejemplo de tu codigo.</t>
         </is>
@@ -855,7 +853,7 @@
           <t>PC</t>
         </is>
       </c>
-      <c r="G15" s="4" t="inlineStr">
+      <c r="G15" s="3" t="inlineStr">
         <is>
           <t>T01 recibida, pero faltan los tres .class y dejaste dentro de los comentarios y del quiz las preguntas de la plantilla (los parentesis con instrucciones). Borralos y sube los .class.</t>
         </is>
@@ -889,10 +887,10 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G16" s="4" t="inlineStr">
+          <t>NP</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
         <is>
           <t>Tu P02 sigue sin compilar. Falta la P03. Ver tu hoja.</t>
         </is>
@@ -926,10 +924,10 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G17" s="4" t="inlineStr">
+          <t>NP</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
         <is>
           <t>Tu HolaMundo no lleva tu nombre. Faltan la P02 y la P03.</t>
         </is>
@@ -963,10 +961,10 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G18" s="4" t="inlineStr">
+          <t>NP</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
         <is>
           <t>Ya llego tu primera entrega. Faltan la P01, la P02 y la P03.</t>
         </is>
@@ -1000,10 +998,10 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G19" s="4" t="inlineStr">
+          <t>NP</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
         <is>
           <t>P03 recibida y con 35 de 36 aciertos, pero falta el documento con las explicaciones y tu carpeta esta escrita 'hermenegilo_eduardo', sin la d. Renombrala a hermenegildo_eduardo.</t>
         </is>
@@ -1038,7 +1036,7 @@
       <c r="F20" t="n">
         <v>9</v>
       </c>
-      <c r="G20" s="4" t="inlineStr">
+      <c r="G20" s="3" t="inlineStr">
         <is>
           <t>T01 completa y corriendo. Detalles: los tres programas imprimen 'RADIOGRAFIA: MiObjeto', que es el titulo de la plantilla, y a dos comentarios les falta la linea QUE IGNORE.</t>
         </is>
@@ -1073,7 +1071,7 @@
       <c r="F21" t="n">
         <v>10</v>
       </c>
-      <c r="G21" s="4" t="inlineStr">
+      <c r="G21" s="3" t="inlineStr">
         <is>
           <t>T01 impecable: los tres .class corren, el modelado justifica cada atributo y metodo, y el quiz usa ejemplos de tu propio codigo.</t>
         </is>
@@ -1107,10 +1105,10 @@
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G22" s="4" t="inlineStr">
+          <t>NP</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
         <is>
           <t>Tu P03 esta completa y bien explicada. Detalle: en tu comentario del 7.2 escribiste 'primo' donde querias decir 'par'.</t>
         </is>
@@ -1145,7 +1143,7 @@
       <c r="F23" t="n">
         <v>9</v>
       </c>
-      <c r="G23" s="4" t="inlineStr">
+      <c r="G23" s="3" t="inlineStr">
         <is>
           <t>T01 completa y corriendo. Un detalle: la subiste a entregas/hernandez_emily/t01/ y va en entregas/hernandez_emily/tareas/t01/.</t>
         </is>
@@ -1182,7 +1180,7 @@
           <t>PC</t>
         </is>
       </c>
-      <c r="G24" s="4" t="inlineStr">
+      <c r="G24" s="3" t="inlineStr">
         <is>
           <t>El mejor analisis del grupo, aceptada. Para que lo tengas: tu 7.2 imprime true y se pedia false, y tu documento no trae tu nombre. T01: le falta casi todo lo que se califica: comentario de modelado, etiquetas, firmas, los .class, tipos y varios operadores. Ver tu hoja.</t>
         </is>
@@ -1219,7 +1217,7 @@
           <t>PC</t>
         </is>
       </c>
-      <c r="G25" s="4" t="inlineStr">
+      <c r="G25" s="3" t="inlineStr">
         <is>
           <t>T01 recibida, pero faltan los tres .class, el quiz debe llamarse QUIZ.md (subiste 'Quiz de la T01.txt'), la carpeta va en minusculas (tareas/t01) y ningun metodo trae su '// firma:'.</t>
         </is>
@@ -1253,10 +1251,10 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G26" s="4" t="inlineStr">
+          <t>NP</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
         <is>
           <t>Aceptada tu P03 en 8 (ver tu hoja). Llegaron tu P01, que esta bien, y tu P02, que no compila: tambien en tu hoja.</t>
         </is>
@@ -1290,10 +1288,10 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G27" s="4" t="inlineStr">
+          <t>NP</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
         <is>
           <t>Tu bloque 7 esta completo y eres el unico que puso el comentario del operador en cada linea. Falto la captura de la TABLA FINAL, que era lo que se pedia, y tu analisis va por temas en vez de falla por falla.</t>
         </is>
@@ -1325,10 +1323,10 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G28" s="4" t="inlineStr">
+          <t>NP</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
         <is>
           <t>P03 lista: tabla completa y el mejor analisis del grupo, con tus palabras. Dos cosas de orden: tu carpeta se llama diego_mendez y deberia ser mendez_juan, donde estan tu P00 y P01, y tienes dos ramas de entregas; trabaja solo en entregas_mendez_juan.</t>
         </is>
@@ -1362,10 +1360,10 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G29" s="4" t="inlineStr">
+          <t>NP</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
         <is>
           <t>Sin entregas registradas.</t>
         </is>
@@ -1402,7 +1400,7 @@
           <t>9</t>
         </is>
       </c>
-      <c r="G30" s="4" t="inlineStr">
+      <c r="G30" s="3" t="inlineStr">
         <is>
           <t>Entrega correcta y completa. T01: 9. Tus clases, tu modelado y tu QUIZ estan bien; entre las tres faltaron la resta, la division, el %, un abreviado, un segundo relacional y un logico.</t>
         </is>
@@ -1439,7 +1437,7 @@
           <t>PC</t>
         </is>
       </c>
-      <c r="G31" s="4" t="inlineStr">
+      <c r="G31" s="3" t="inlineStr">
         <is>
           <t>Sigue igual que el 14-sep: tu T01 esta completa (compila y el quiz tiene las 10 respuestas) pero vive en entregas/Paula_Romero/, suelta y sin .class. Muevela a entregas/romero_paula/tareas/t01/, agrega los .class y mueve tambien la P03.</t>
         </is>
@@ -1476,7 +1474,7 @@
           <t>PC</t>
         </is>
       </c>
-      <c r="G32" s="4" t="inlineStr">
+      <c r="G32" s="3" t="inlineStr">
         <is>
           <t>T01 recibida, pero faltan los tres .class, el quiz solo trae 2 de las 10 respuestas y subiste MiObjeto.java, que es la plantilla sin llenar.</t>
         </is>
@@ -1513,7 +1511,7 @@
           <t>9</t>
         </is>
       </c>
-      <c r="G33" s="4" t="inlineStr">
+      <c r="G33" s="3" t="inlineStr">
         <is>
           <t>Incompleta: en tu carpeta solo esta el Laboratorio.class. Aunque el trabajo sea de equipo, cada quien sube su .java y su documento con la captura y el analisis. Ver tu hoja. T01: 9, pero esta en una rama suelta: pasala a tu rama del semestre (ver tu hoja). Entre tus clases faltaron la suma, la resta y la division como operadores aritmeticos.</t>
         </is>
@@ -1550,7 +1548,7 @@
           <t>8</t>
         </is>
       </c>
-      <c r="G34" s="4" t="inlineStr">
+      <c r="G34" s="3" t="inlineStr">
         <is>
           <t>Tu P03 sigue sin estar en tu carpeta: ver tu hoja. T01: 8. Tus operadores estan completos, pero tus atributos no estan etiquetados, no escribiste las firmas, tu main no separa estado inicial, invocaciones y estado final, y Raqueta no tiene un metodo void con parametro. Ademas la subiste a una rama suelta: ver tu hoja.</t>
         </is>
@@ -1587,50 +1585,47 @@
           <t>PC</t>
         </is>
       </c>
-      <c r="G35" s="4" t="inlineStr">
+      <c r="G35" s="3" t="inlineStr">
         <is>
           <t>T01 recibida, pero faltan los tres .class y a los tres comentarios de modelado les falta la linea QUE IGNORE.</t>
         </is>
       </c>
     </row>
-    <row r="36"/>
-    <row r="37"/>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>P00:  calificadas 27   ·   pendientes de correccion 0   ·   sin entregar 2</t>
+          <t>P00:  calificadas 27   ·   pendientes de correccion 0   ·   no entregadas 2</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>P01:  calificadas 26   ·   pendientes de correccion 0   ·   sin entregar 3</t>
+          <t>P01:  calificadas 26   ·   pendientes de correccion 0   ·   no entregadas 3</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>P02:  calificadas 21   ·   pendientes de correccion 2   ·   sin entregar 6</t>
+          <t>P02:  calificadas 21   ·   pendientes de correccion 2   ·   no entregadas 6</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>P03:  calificadas 18   ·   pendientes de correccion 5   ·   sin entregar 6</t>
+          <t>P03:  calificadas 18   ·   pendientes de correccion 5   ·   no entregadas 6</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>T01:  calificadas 9   ·   pendientes de correccion 8   ·   sin entregar 12</t>
-        </is>
-      </c>
-    </row>
-    <row r="43"/>
+          <t>T01:  calificadas 9   ·   pendientes de correccion 8   ·   no entregadas 12</t>
+        </is>
+      </c>
+    </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
@@ -1652,8 +1647,8 @@
   <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="62" customWidth="1" style="2" min="1" max="1"/>
-    <col width="72" customWidth="1" style="2" min="2" max="2"/>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1671,51 +1666,50 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>P00: 10    P01: NP    P02: NP    P03: NP    T01: —</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Ya llego tu primera entrega. Faltan la P01, la P02 y la P03.</t>
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Tu P00 quedo en una rama suelta (Shagr33l-patch-1) y no cuenta.</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Copiala a entregas/gutierrez_ixcmie/p00/ en tu rama entregas_gutierrez_ixcmie.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Faltan P01, P02, P03 y T01.</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>Subelas en sus carpetas de tu rama.</t>
         </is>
@@ -1735,8 +1729,8 @@
   <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="62" customWidth="1" style="2" min="1" max="1"/>
-    <col width="72" customWidth="1" style="2" min="2" max="2"/>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1754,63 +1748,62 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>P00: 10    P01: 10    P02: NP    P03: PC    T01: —</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>P03 recibida y con 35 de 36 aciertos, pero falta el documento con las explicaciones y tu carpeta esta escrita 'hermenegilo_eduardo', sin la d. Renombrala a hermenegildo_eduardo.</t>
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Tu carpeta se llama hermenegilo_eduardo, sin la d.</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Renombrala a hermenegildo_eduardo para que quede junto a tu P00 y P01.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Falta el documento con las explicaciones de la P03.</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>Explica por que fallaste cada expresion; acertaste 35 de 36, asi que es corto.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>Falta la T01.</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>3 .java, 3 .class y QUIZ.md en tareas/t01/.</t>
         </is>
@@ -1830,8 +1823,8 @@
   <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="62" customWidth="1" style="2" min="1" max="1"/>
-    <col width="72" customWidth="1" style="2" min="2" max="2"/>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1849,39 +1842,38 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>P00: 10    P01: 9    P02: 10    P03: 10    T01: —</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Tu P03 esta completa y bien explicada. Detalle: en tu comentario del 7.2 escribiste 'primo' donde querias decir 'par'.</t>
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Falta la T01.</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Tu rama t01-HernandezGonzalez solo tiene practicas viejas. Sube la tarea en entregas/hernandez_mauricio/tareas/t01/, en tu rama entregas_hernandez_mauricio.</t>
         </is>
@@ -1901,8 +1893,8 @@
   <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="62" customWidth="1" style="2" min="1" max="1"/>
-    <col width="72" customWidth="1" style="2" min="2" max="2"/>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1920,51 +1912,50 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>P00: 10    P01: 10    P02: 10    P03: 10    T01: 9</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>T01 completa y corriendo. Detalles: los tres programas imprimen 'RADIOGRAFIA: MiObjeto', que es el titulo de la plantilla, y a dos comentarios les falta la linea QUE IGNORE.</t>
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Los tres programas imprimen 'RADIOGRAFIA: MiObjeto'.</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Cambia ese titulo por el nombre real de cada clase.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>A dos comentarios les falta la linea QUE IGNORE.</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>Agregala: una o dos cosas del objeto real que no modelaste, y por que.</t>
         </is>
@@ -1984,8 +1975,8 @@
   <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="62" customWidth="1" style="2" min="1" max="1"/>
-    <col width="72" customWidth="1" style="2" min="2" max="2"/>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2003,39 +1994,38 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>P00: 10    P01: 10    P02: 9    P03: 10    T01: 9</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>T01 completa y corriendo. Un detalle: la subiste a entregas/hernandez_emily/t01/ y va en entregas/hernandez_emily/tareas/t01/.</t>
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Tu T01 esta en entregas/hernandez_emily/t01/.</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Muevela a entregas/hernandez_emily/tareas/t01/, que es la ruta del enunciado.</t>
         </is>
@@ -2055,8 +2045,8 @@
   <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="62" customWidth="1" style="2" min="1" max="1"/>
-    <col width="72" customWidth="1" style="2" min="2" max="2"/>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2074,39 +2064,38 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>P00: 10    P01: 9    P02: 9    P03: 10    T01: PC</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>El mejor analisis del grupo, aceptada. Para que lo tengas: tu 7.2 imprime true y se pedia false, y tu documento no trae tu nombre. T01: le falta casi todo lo que se califica: comentario de modelado, etiquetas, firmas, los .class, tipos y varios operadores. Ver tu hoja.</t>
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Sigue pendiente lo del 14-sep.</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Revisa la observacion de tu corte anterior y sube el arreglo; avisame cuando este.</t>
         </is>
@@ -2126,8 +2115,8 @@
   <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="62" customWidth="1" style="2" min="1" max="1"/>
-    <col width="72" customWidth="1" style="2" min="2" max="2"/>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2145,75 +2134,74 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>P00: 10    P01: 10    P02: 9    P03: 9    T01: PC</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>T01 recibida, pero faltan los tres .class, el quiz debe llamarse QUIZ.md (subiste 'Quiz de la T01.txt'), la carpeta va en minusculas (tareas/t01) y ningun metodo trae su '// firma:'.</t>
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Tu T01 no trae los .class.</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Compila los tres con JDK 21 y subelos.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>El quiz se llama 'Quiz de la T01.txt'.</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>Debe ser QUIZ.md.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>Tu carpeta es Tareas/T01, con mayusculas.</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>Usa tareas/t01 en minusculas.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>Ningun metodo trae su firma en comentario.</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>Agrega // firma: metodo(tipo) arriba de cada metodo.</t>
         </is>
@@ -2233,8 +2221,8 @@
   <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="62" customWidth="1" style="2" min="1" max="1"/>
-    <col width="72" customWidth="1" style="2" min="2" max="2"/>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2252,51 +2240,50 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>P00: 10    P01: 10    P02: PC    P03: 8    T01: —</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Aceptada tu P03 en 8 (ver tu hoja). Llegaron tu P01, que esta bien, y tu P02, que no compila: tambien en tu hoja.</t>
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Tu P02 sigue pendiente desde el 14-sep.</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Revisa la observacion anterior y sube el arreglo.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Falta la T01.</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>3 .java, 3 .class y QUIZ.md en tareas/t01/.</t>
         </is>
@@ -2316,8 +2303,8 @@
   <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="62" customWidth="1" style="2" min="1" max="1"/>
-    <col width="72" customWidth="1" style="2" min="2" max="2"/>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2335,39 +2322,38 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>P00: 10    P01: 10    P02: 10    P03: 9    T01: —</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Tu bloque 7 esta completo y eres el unico que puso el comentario del operador en cada linea. Falto la captura de la TABLA FINAL, que era lo que se pedia, y tu analisis va por temas en vez de falla por falla.</t>
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Falta la T01.</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>3 .java, 3 .class y QUIZ.md en entregas/medina_miguel/tareas/t01/.</t>
         </is>
@@ -2387,8 +2373,8 @@
   <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="62" customWidth="1" style="2" min="1" max="1"/>
-    <col width="72" customWidth="1" style="2" min="2" max="2"/>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2406,63 +2392,62 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>P00: 10    P01: 9    P02: 10    P03: 10    T01: —</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>P03 lista: tabla completa y el mejor analisis del grupo, con tus palabras. Dos cosas de orden: tu carpeta se llama diego_mendez y deberia ser mendez_juan, donde estan tu P00 y P01, y tienes dos ramas de entregas; trabaja solo en entregas_mendez_juan.</t>
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Tu carpeta se llama diego_mendez.</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Deberia ser mendez_juan, donde estan tu P00 y tu P01.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Tienes dos ramas de entregas.</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>Trabaja solo en entregas_mendez_juan; la otra ya no la uses.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>Falta la T01.</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>3 .java, 3 .class y QUIZ.md en tareas/t01/.</t>
         </is>
@@ -2482,8 +2467,8 @@
   <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="62" customWidth="1" style="2" min="1" max="1"/>
-    <col width="72" customWidth="1" style="2" min="2" max="2"/>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2501,39 +2486,38 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>P00: 10    P01: 9    P02: 10    P03: 10    T01: —</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>P03 lista: tabla completa y analisis en el PDF (documento conjunto con otros dos companeros). En mis-resultados.txt dejaste en blanco los 'por que me equivoque', pero estan explicados en el PDF. Falta la T01.</t>
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Falta la T01 completa.</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Sube los 3 .java, sus 3 .class y QUIZ.md en entregas/ajas_andre/tareas/t01/.</t>
         </is>
@@ -2553,8 +2537,8 @@
   <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="62" customWidth="1" style="2" min="1" max="1"/>
-    <col width="72" customWidth="1" style="2" min="2" max="2"/>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2572,39 +2556,38 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>P00: NP    P01: NP    P02: NP    P03: NP    T01: —</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Sin entregas registradas.</t>
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>No hay ninguna entrega tuya en el repo.</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Crea tu rama entregas_olmedo_marco y sube P00, P01, P02 y P03; despues la T01.</t>
         </is>
@@ -2624,8 +2607,8 @@
   <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="62" customWidth="1" style="2" min="1" max="1"/>
-    <col width="72" customWidth="1" style="2" min="2" max="2"/>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2643,51 +2626,50 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>P00: 10    P01: 9    P02: 10    P03: PC    T01: PC</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Sigue igual que el 14-sep: tu T01 esta completa (compila y el quiz tiene las 10 respuestas) pero vive en entregas/Paula_Romero/, suelta y sin .class. Muevela a entregas/romero_paula/tareas/t01/, agrega los .class y mueve tambien la P03.</t>
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Tu T01 esta completa pero suelta en entregas/Paula_Romero/.</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Muevela a entregas/romero_paula/tareas/t01/ y agrega los tres .class; tu codigo ya compila con JDK 21.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Tu P03 tambien esta en esa carpeta.</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>Muevela a entregas/romero_paula/p03/.</t>
         </is>
@@ -2707,8 +2689,8 @@
   <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="62" customWidth="1" style="2" min="1" max="1"/>
-    <col width="72" customWidth="1" style="2" min="2" max="2"/>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2726,75 +2708,74 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>P00: 10    P01: 9    P02: 10    P03: PC    T01: PC</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>T01 recibida, pero faltan los tres .class, el quiz solo trae 2 de las 10 respuestas y subiste MiObjeto.java, que es la plantilla sin llenar.</t>
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Tu T01 no trae los .class.</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Compila los tres con JDK 21 y subelos.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>El quiz solo tiene 2 de las 10 respuestas.</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>Completa las otras ocho, con tus palabras.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>Subiste MiObjeto.java, que es la plantilla sin llenar.</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>Borrala de tu carpeta.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>Tu P03 sigue pendiente desde el 14-sep.</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>Revisa la observacion anterior y sube el arreglo.</t>
         </is>
@@ -2814,8 +2795,8 @@
   <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="62" customWidth="1" style="2" min="1" max="1"/>
-    <col width="72" customWidth="1" style="2" min="2" max="2"/>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2833,39 +2814,38 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>P00: 10    P01: 10    P02: 10    P03: PC    T01: 9</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Incompleta: en tu carpeta solo esta el Laboratorio.class. Aunque el trabajo sea de equipo, cada quien sube su .java y su documento con la captura y el analisis. Ver tu hoja. T01: 9, pero esta en una rama suelta: pasala a tu rama del semestre (ver tu hoja). Entre tus clases faltaron la suma, la resta y la division como operadores aritmeticos.</t>
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>En tu p03 solo esta Laboratorio.class.</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Sube tambien Laboratorio.java y mis-resultados.txt con tu tabla.</t>
         </is>
@@ -2885,8 +2865,8 @@
   <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="62" customWidth="1" style="2" min="1" max="1"/>
-    <col width="72" customWidth="1" style="2" min="2" max="2"/>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2904,39 +2884,38 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>P00: 10    P01: 10    P02: 10    P03: PC    T01: 8</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Tu P03 sigue sin estar en tu carpeta: ver tu hoja. T01: 8. Tus operadores estan completos, pero tus atributos no estan etiquetados, no escribiste las firmas, tu main no separa estado inicial, invocaciones y estado final, y Raqueta no tiene un metodo void con parametro. Ademas la subiste a una rama suelta: ver tu hoja.</t>
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Tu P03 sigue pendiente desde el 14-sep.</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Revisa la observacion anterior y sube el arreglo.</t>
         </is>
@@ -2956,8 +2935,8 @@
   <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="62" customWidth="1" style="2" min="1" max="1"/>
-    <col width="72" customWidth="1" style="2" min="2" max="2"/>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2975,51 +2954,50 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>P00: 10    P01: 10    P02: 10    P03: 9    T01: PC</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>T01 recibida, pero faltan los tres .class y a los tres comentarios de modelado les falta la linea QUE IGNORE.</t>
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Tu T01 no trae los .class.</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Compila los tres con JDK 21 y subelos.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>A los tres comentarios les falta la linea QUE IGNORE.</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>Agregala en cada clase.</t>
         </is>
@@ -3039,8 +3017,8 @@
   <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="62" customWidth="1" style="2" min="1" max="1"/>
-    <col width="72" customWidth="1" style="2" min="2" max="2"/>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3058,39 +3036,38 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>P00: 10    P01: 10    P02: 10    P03: 10    T01: PC</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Tu T01 quedo sin los .class: los borraste el 21-sep. El codigo compila bien con JDK 21 y el modelado y el quiz estan muy completos; recompila los tres y subelos para cerrarla.</t>
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Borraste tus tres .class el 21-sep, y la T01 se califica ejecutandolos.</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Compila con el JDK 21 (javac Bicicleta.java, etc.), pruebalo con java Bicicleta y sube los tres .class junto a tus .java.</t>
         </is>
@@ -3110,8 +3087,8 @@
   <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="62" customWidth="1" style="2" min="1" max="1"/>
-    <col width="72" customWidth="1" style="2" min="2" max="2"/>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3129,51 +3106,50 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>P00: 10    P01: 10    P02: NP    P03: NP    T01: —</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Faltan la P02 y la P03.</t>
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>No tienes P02 ni P03.</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Sube la P02 en entregas/castillo_ihsahn/p02/ y la P03 en p03/, con Laboratorio.java y mis-resultados.txt.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Falta la T01.</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>3 .java, 3 .class y QUIZ.md en tareas/t01/.</t>
         </is>
@@ -3193,8 +3169,8 @@
   <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="62" customWidth="1" style="2" min="1" max="1"/>
-    <col width="72" customWidth="1" style="2" min="2" max="2"/>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3212,51 +3188,50 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>P00: 10    P01: 10    P02: 10    P03: 10    T01: PC</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>P03 lista: tabla de 41 filas con analisis en PDF y captura. En la T01 faltan los tres .class y ningun metodo trae su '// firma:' en comentario.</t>
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Tu T01 no trae los .class.</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Compila los tres con JDK 21 y subelos.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Ningun metodo trae su firma en comentario.</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>Agrega // firma: metodo(tipo) arriba de cada metodo, como pide el enunciado.</t>
         </is>
@@ -3276,8 +3251,8 @@
   <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="62" customWidth="1" style="2" min="1" max="1"/>
-    <col width="72" customWidth="1" style="2" min="2" max="2"/>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3295,39 +3270,38 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>P00: NP    P01: NP    P02: NP    P03: NP    T01: —</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Sin entregas registradas.</t>
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>No hay ninguna entrega tuya en el repo.</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Crea tu rama entregas_cruz_isaac y sube P00, P01, P02 y P03; despues la T01.</t>
         </is>
@@ -3347,8 +3321,8 @@
   <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="62" customWidth="1" style="2" min="1" max="1"/>
-    <col width="72" customWidth="1" style="2" min="2" max="2"/>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3366,51 +3340,50 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>P00: 10    P01: 10    P02: 10    P03: 10    T01: PC</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>T01 recibida, pero faltan los tres .class y dejaste dentro de los comentarios y del quiz las preguntas de la plantilla (los parentesis con instrucciones). Borralos y sube los .class.</t>
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Tu T01 no trae los .class.</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Compila los tres con JDK 21 y subelos.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Dejaste las preguntas de la plantilla dentro de los comentarios y del quiz.</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>Borra los parentesis con las instrucciones y deja solo tu respuesta.</t>
         </is>
@@ -3430,8 +3403,8 @@
   <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="62" customWidth="1" style="2" min="1" max="1"/>
-    <col width="72" customWidth="1" style="2" min="2" max="2"/>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3449,51 +3422,50 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>P00: 10    P01: 10    P02: PC    P03: NP    T01: —</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Tu P02 sigue sin compilar. Falta la P03. Ver tu hoja.</t>
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Tu P02 no compila.</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Arregla PruebaPunto para que corra y vuelve a subirla.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>No tienes P03 ni T01.</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>Sube la P03 en p03/ y la T01 en tareas/t01/.</t>
         </is>
@@ -3513,8 +3485,8 @@
   <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="62" customWidth="1" style="2" min="1" max="1"/>
-    <col width="72" customWidth="1" style="2" min="2" max="2"/>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3532,39 +3504,38 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>P00: 10    P01: 9    P02: NP    P03: NP    T01: —</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Tu HolaMundo no lleva tu nombre. Faltan la P02 y la P03.</t>
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>No tienes P02, P03 ni T01.</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Sube cada una en su carpeta dentro de entregas/gonzalez_ramon/.</t>
         </is>

</xml_diff>

<commit_message>
Corte 21-sep: NP en la T01 sin entregar y la T01 recibida por correo, calificada
</commit_message>
<xml_diff>
--- a/calificaciones/P00-T01-corte-21sep.xlsx
+++ b/calificaciones/P00-T01-corte-21sep.xlsx
@@ -1103,14 +1103,12 @@
           <t>10</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>NP</t>
-        </is>
+      <c r="F22" t="n">
+        <v>8</v>
       </c>
       <c r="G22" s="3" t="inlineStr">
         <is>
-          <t>Tu P03 esta completa y bien explicada. Detalle: en tu comentario del 7.2 escribiste 'primo' donde querias decir 'par'.</t>
+          <t>T01 entregada por correo, no por Git: dice que creo las ramas pero no lo dejo hacer push. Los .class corren con JDK 21 y el quiz trae las 10 respuestas con tus palabras. Le falta el comentario de modelado en las cuatro lineas etiquetadas, el '// firma:' de cada metodo y que cada objeto tenga su propio main; por eso 8. Falta subirla a entregas/hernandez_mauricio/tareas/t01/.</t>
         </is>
       </c>
     </row>
@@ -1622,14 +1620,14 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>T01:  calificadas 9   ·   pendientes de correccion 8   ·   no entregadas 12</t>
+          <t>T01:  calificadas 10   ·   pendientes de correccion 8   ·   no entregadas 11</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Cambios desde el 14-sep: se calificaron 3 P03 nuevas y 4 T01 nuevas. Otras 6 T01 llegaron completas pero quedaron pendientes porque les faltan los .class; su codigo compila con JDK 21.</t>
+          <t>Cambios desde el 14-sep: 4 T01 nuevas calificadas, una mas recibida por correo, y 3 P03 nuevas. Seis T01 quedan pendientes solo porque les faltan los .class; su codigo compila con JDK 21.</t>
         </is>
       </c>
     </row>
@@ -1820,7 +1818,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="62" customWidth="1" min="1" max="1"/>
@@ -1844,14 +1842,14 @@
     <row r="3">
       <c r="A3" s="4" t="inlineStr">
         <is>
-          <t>P00: 10    P01: 9    P02: 10    P03: 10    T01: —</t>
+          <t>P00: 10    P01: 9    P02: 10    P03: 10    T01: 8</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="3" t="inlineStr">
         <is>
-          <t>Tu P03 esta completa y bien explicada. Detalle: en tu comentario del 7.2 escribiste 'primo' donde querias decir 'par'.</t>
+          <t>T01 entregada por correo, no por Git: dice que creo las ramas pero no lo dejo hacer push. Los .class corren con JDK 21 y el quiz trae las 10 respuestas con tus palabras. Le falta el comentario de modelado en las cuatro lineas etiquetadas, el '// firma:' de cada metodo y que cada objeto tenga su propio main; por eso 8. Falta subirla a entregas/hernandez_mauricio/tareas/t01/.</t>
         </is>
       </c>
     </row>
@@ -1870,12 +1868,48 @@
     <row r="7">
       <c r="A7" s="3" t="inlineStr">
         <is>
-          <t>Falta la T01.</t>
+          <t>Tu T01 llego por correo y no esta en el repo.</t>
         </is>
       </c>
       <c r="B7" s="3" t="inlineStr">
         <is>
-          <t>Tu rama t01-HernandezGonzalez solo tiene practicas viejas. Sube la tarea en entregas/hernandez_mauricio/tareas/t01/, en tu rama entregas_hernandez_mauricio.</t>
+          <t>Subela a entregas/hernandez_mauricio/tareas/t01/ en tu rama entregas_hernandez_mauricio. Si el push sigue fallando, escribeme y lo vemos en un zoom.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Tus comentarios de modelado son prosa corrida.</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Van en cuatro lineas etiquetadas: CONTEXTO, QUE SABE Y POR QUE, QUE SABE HACER Y POR QUE, QUE IGNORE.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Ningun metodo trae su firma en comentario.</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Agrega // firma: metodo(tipo) arriba de cada uno.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Celular no tiene su propio main y dos objetos piden datos por teclado.</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>El enunciado pide que cada objeto tenga su main con estado inicial, invocaciones y estado final, sin Scanner.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Corte 21-sep: T01 sin entregar queda como NP (#86)
* Corte 21-sep: la T01 sin entregar queda como NP

* Corte 21-sep: NP en la T01 sin entregar y la T01 recibida por correo, calificada
</commit_message>
<xml_diff>
--- a/calificaciones/P00-T01-corte-21sep.xlsx
+++ b/calificaciones/P00-T01-corte-21sep.xlsx
@@ -82,10 +82,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -459,13 +458,13 @@
   <dimension ref="A1:G44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="13" customWidth="1" style="2" min="1" max="1"/>
-    <col width="6" customWidth="1" style="2" min="2" max="2"/>
-    <col width="6" customWidth="1" style="2" min="3" max="3"/>
-    <col width="6" customWidth="1" style="2" min="4" max="4"/>
-    <col width="6" customWidth="1" style="2" min="5" max="5"/>
-    <col width="6" customWidth="1" style="2" min="6" max="6"/>
-    <col width="110" customWidth="1" style="2" min="7" max="7"/>
+    <col width="13" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="6" customWidth="1" min="3" max="3"/>
+    <col width="6" customWidth="1" min="4" max="4"/>
+    <col width="6" customWidth="1" min="5" max="5"/>
+    <col width="6" customWidth="1" min="6" max="6"/>
+    <col width="110" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -485,50 +484,49 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>10 = correcta  ·  9 = correcta con un detalle  ·  8 = incompleta pero aceptada  ·  PC = pendiente de correccion (tienes hoja aparte)  ·  NP = no presentada  ·  — = aun no la subes y todavia no vence</t>
+          <t>10 = correcta  ·  9 = correcta con un detalle  ·  8 = incompleta pero aceptada  ·  PC = pendiente de correccion  ·  NP = no entregada al corte</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>P00: el objetivo era demostrar que sabes hacer push, asi que cuenta 10 para todo el que subio algo. T01: vencio el 14-sep; lo entregado hasta el 15-sep cuenta en tiempo por la prorroga que se dio en clase. PC = pendiente de correccion: no es una calificacion final, se recalifica en cuanto subas el arreglo.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5"/>
+          <t>P00: el objetivo era demostrar que sabes hacer push, asi que cuenta 10 para todo el que subio algo. T01: vencio el lunes 14-sep, con la prorroga hasta el final de ese dia que se dio en clase; lo entregado el 15 tambien se conto. NP = no entregada al corte. Si la subes, avisame y la califico: la politica de entregas tardias de MPOO sigue sin definirse.</t>
+        </is>
+      </c>
+    </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Cuenta</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>P00</t>
         </is>
       </c>
-      <c r="C6" s="3" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>P01</t>
         </is>
       </c>
-      <c r="D6" s="3" t="inlineStr">
+      <c r="D6" s="2" t="inlineStr">
         <is>
           <t>P02</t>
         </is>
       </c>
-      <c r="E6" s="3" t="inlineStr">
+      <c r="E6" s="2" t="inlineStr">
         <is>
           <t>P03</t>
         </is>
       </c>
-      <c r="F6" s="3" t="inlineStr">
+      <c r="F6" s="2" t="inlineStr">
         <is>
           <t>T01</t>
         </is>
       </c>
-      <c r="G6" s="3" t="inlineStr">
+      <c r="G6" s="2" t="inlineStr">
         <is>
           <t>Observaciones</t>
         </is>
@@ -560,10 +558,10 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G7" s="4" t="inlineStr">
+          <t>NP</t>
+        </is>
+      </c>
+      <c r="G7" s="3" t="inlineStr">
         <is>
           <t>P03 lista: tabla completa y analisis en el PDF (documento conjunto con otros dos companeros). En mis-resultados.txt dejaste en blanco los 'por que me equivoque', pero estan explicados en el PDF. Falta la T01.</t>
         </is>
@@ -600,7 +598,7 @@
           <t>PC</t>
         </is>
       </c>
-      <c r="G8" s="4" t="inlineStr">
+      <c r="G8" s="3" t="inlineStr">
         <is>
           <t>Tu T01 quedo sin los .class: los borraste el 21-sep. El codigo compila bien con JDK 21 y el modelado y el quiz estan muy completos; recompila los tres y subelos para cerrarla.</t>
         </is>
@@ -637,7 +635,7 @@
           <t>10</t>
         </is>
       </c>
-      <c r="G9" s="4" t="inlineStr">
+      <c r="G9" s="3" t="inlineStr">
         <is>
           <t>Bloque 7 completo y buen analisis; tu captura no muestra la tabla final, solo el final del reporte. Tu T01 esta muy bien: 10. Dos detalles para la proxima: a Television le falto la linea QUE IGNORE, y entre las tres clases no usaste la resta.</t>
         </is>
@@ -671,10 +669,10 @@
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G10" s="4" t="inlineStr">
+          <t>NP</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr">
         <is>
           <t>Faltan la P02 y la P03.</t>
         </is>
@@ -709,7 +707,7 @@
           <t>PC</t>
         </is>
       </c>
-      <c r="G11" s="4" t="inlineStr">
+      <c r="G11" s="3" t="inlineStr">
         <is>
           <t>P03 lista: tabla de 41 filas con analisis en PDF y captura. En la T01 faltan los tres .class y ningun metodo trae su '// firma:' en comentario.</t>
         </is>
@@ -744,7 +742,7 @@
       <c r="F12" t="n">
         <v>10</v>
       </c>
-      <c r="G12" s="4" t="inlineStr">
+      <c r="G12" s="3" t="inlineStr">
         <is>
           <t>T01 completa: los tres .class corren, el modelado tiene contexto propio y el quiz esta con tus palabras.</t>
         </is>
@@ -778,10 +776,10 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G13" s="4" t="inlineStr">
+          <t>NP</t>
+        </is>
+      </c>
+      <c r="G13" s="3" t="inlineStr">
         <is>
           <t>Sin entregas registradas.</t>
         </is>
@@ -818,7 +816,7 @@
           <t>9</t>
         </is>
       </c>
-      <c r="G14" s="4" t="inlineStr">
+      <c r="G14" s="3" t="inlineStr">
         <is>
           <t>Completa. Detalle: tu explicacion del desbordamiento de Integer.MAX_VALUE quedo confusa. T01: 9. Te falto el operador %, MiCuaderno no tiene un metodo void con parametro y en el QUIZ la pregunta 1 no trae ejemplo de tu codigo.</t>
         </is>
@@ -855,7 +853,7 @@
           <t>PC</t>
         </is>
       </c>
-      <c r="G15" s="4" t="inlineStr">
+      <c r="G15" s="3" t="inlineStr">
         <is>
           <t>T01 recibida, pero faltan los tres .class y dejaste dentro de los comentarios y del quiz las preguntas de la plantilla (los parentesis con instrucciones). Borralos y sube los .class.</t>
         </is>
@@ -889,10 +887,10 @@
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G16" s="4" t="inlineStr">
+          <t>NP</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
         <is>
           <t>Tu P02 sigue sin compilar. Falta la P03. Ver tu hoja.</t>
         </is>
@@ -926,10 +924,10 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G17" s="4" t="inlineStr">
+          <t>NP</t>
+        </is>
+      </c>
+      <c r="G17" s="3" t="inlineStr">
         <is>
           <t>Tu HolaMundo no lleva tu nombre. Faltan la P02 y la P03.</t>
         </is>
@@ -963,10 +961,10 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G18" s="4" t="inlineStr">
+          <t>NP</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
         <is>
           <t>Ya llego tu primera entrega. Faltan la P01, la P02 y la P03.</t>
         </is>
@@ -1000,10 +998,10 @@
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G19" s="4" t="inlineStr">
+          <t>NP</t>
+        </is>
+      </c>
+      <c r="G19" s="3" t="inlineStr">
         <is>
           <t>P03 recibida y con 35 de 36 aciertos, pero falta el documento con las explicaciones y tu carpeta esta escrita 'hermenegilo_eduardo', sin la d. Renombrala a hermenegildo_eduardo.</t>
         </is>
@@ -1038,7 +1036,7 @@
       <c r="F20" t="n">
         <v>9</v>
       </c>
-      <c r="G20" s="4" t="inlineStr">
+      <c r="G20" s="3" t="inlineStr">
         <is>
           <t>T01 completa y corriendo. Detalles: los tres programas imprimen 'RADIOGRAFIA: MiObjeto', que es el titulo de la plantilla, y a dos comentarios les falta la linea QUE IGNORE.</t>
         </is>
@@ -1073,7 +1071,7 @@
       <c r="F21" t="n">
         <v>10</v>
       </c>
-      <c r="G21" s="4" t="inlineStr">
+      <c r="G21" s="3" t="inlineStr">
         <is>
           <t>T01 impecable: los tres .class corren, el modelado justifica cada atributo y metodo, y el quiz usa ejemplos de tu propio codigo.</t>
         </is>
@@ -1105,14 +1103,12 @@
           <t>10</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G22" s="4" t="inlineStr">
-        <is>
-          <t>Tu P03 esta completa y bien explicada. Detalle: en tu comentario del 7.2 escribiste 'primo' donde querias decir 'par'.</t>
+      <c r="F22" t="n">
+        <v>8</v>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>T01 entregada por correo, no por Git: dice que creo las ramas pero no lo dejo hacer push. Los .class corren con JDK 21 y el quiz trae las 10 respuestas con tus palabras. Le falta el comentario de modelado en las cuatro lineas etiquetadas, el '// firma:' de cada metodo y que cada objeto tenga su propio main; por eso 8. Falta subirla a entregas/hernandez_mauricio/tareas/t01/.</t>
         </is>
       </c>
     </row>
@@ -1145,7 +1141,7 @@
       <c r="F23" t="n">
         <v>9</v>
       </c>
-      <c r="G23" s="4" t="inlineStr">
+      <c r="G23" s="3" t="inlineStr">
         <is>
           <t>T01 completa y corriendo. Un detalle: la subiste a entregas/hernandez_emily/t01/ y va en entregas/hernandez_emily/tareas/t01/.</t>
         </is>
@@ -1182,7 +1178,7 @@
           <t>PC</t>
         </is>
       </c>
-      <c r="G24" s="4" t="inlineStr">
+      <c r="G24" s="3" t="inlineStr">
         <is>
           <t>El mejor analisis del grupo, aceptada. Para que lo tengas: tu 7.2 imprime true y se pedia false, y tu documento no trae tu nombre. T01: le falta casi todo lo que se califica: comentario de modelado, etiquetas, firmas, los .class, tipos y varios operadores. Ver tu hoja.</t>
         </is>
@@ -1219,7 +1215,7 @@
           <t>PC</t>
         </is>
       </c>
-      <c r="G25" s="4" t="inlineStr">
+      <c r="G25" s="3" t="inlineStr">
         <is>
           <t>T01 recibida, pero faltan los tres .class, el quiz debe llamarse QUIZ.md (subiste 'Quiz de la T01.txt'), la carpeta va en minusculas (tareas/t01) y ningun metodo trae su '// firma:'.</t>
         </is>
@@ -1253,10 +1249,10 @@
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G26" s="4" t="inlineStr">
+          <t>NP</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
         <is>
           <t>Aceptada tu P03 en 8 (ver tu hoja). Llegaron tu P01, que esta bien, y tu P02, que no compila: tambien en tu hoja.</t>
         </is>
@@ -1290,10 +1286,10 @@
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G27" s="4" t="inlineStr">
+          <t>NP</t>
+        </is>
+      </c>
+      <c r="G27" s="3" t="inlineStr">
         <is>
           <t>Tu bloque 7 esta completo y eres el unico que puso el comentario del operador en cada linea. Falto la captura de la TABLA FINAL, que era lo que se pedia, y tu analisis va por temas en vez de falla por falla.</t>
         </is>
@@ -1325,10 +1321,10 @@
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G28" s="4" t="inlineStr">
+          <t>NP</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
         <is>
           <t>P03 lista: tabla completa y el mejor analisis del grupo, con tus palabras. Dos cosas de orden: tu carpeta se llama diego_mendez y deberia ser mendez_juan, donde estan tu P00 y P01, y tienes dos ramas de entregas; trabaja solo en entregas_mendez_juan.</t>
         </is>
@@ -1362,10 +1358,10 @@
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="G29" s="4" t="inlineStr">
+          <t>NP</t>
+        </is>
+      </c>
+      <c r="G29" s="3" t="inlineStr">
         <is>
           <t>Sin entregas registradas.</t>
         </is>
@@ -1402,7 +1398,7 @@
           <t>9</t>
         </is>
       </c>
-      <c r="G30" s="4" t="inlineStr">
+      <c r="G30" s="3" t="inlineStr">
         <is>
           <t>Entrega correcta y completa. T01: 9. Tus clases, tu modelado y tu QUIZ estan bien; entre las tres faltaron la resta, la division, el %, un abreviado, un segundo relacional y un logico.</t>
         </is>
@@ -1439,7 +1435,7 @@
           <t>PC</t>
         </is>
       </c>
-      <c r="G31" s="4" t="inlineStr">
+      <c r="G31" s="3" t="inlineStr">
         <is>
           <t>Sigue igual que el 14-sep: tu T01 esta completa (compila y el quiz tiene las 10 respuestas) pero vive en entregas/Paula_Romero/, suelta y sin .class. Muevela a entregas/romero_paula/tareas/t01/, agrega los .class y mueve tambien la P03.</t>
         </is>
@@ -1476,7 +1472,7 @@
           <t>PC</t>
         </is>
       </c>
-      <c r="G32" s="4" t="inlineStr">
+      <c r="G32" s="3" t="inlineStr">
         <is>
           <t>T01 recibida, pero faltan los tres .class, el quiz solo trae 2 de las 10 respuestas y subiste MiObjeto.java, que es la plantilla sin llenar.</t>
         </is>
@@ -1513,7 +1509,7 @@
           <t>9</t>
         </is>
       </c>
-      <c r="G33" s="4" t="inlineStr">
+      <c r="G33" s="3" t="inlineStr">
         <is>
           <t>Incompleta: en tu carpeta solo esta el Laboratorio.class. Aunque el trabajo sea de equipo, cada quien sube su .java y su documento con la captura y el analisis. Ver tu hoja. T01: 9, pero esta en una rama suelta: pasala a tu rama del semestre (ver tu hoja). Entre tus clases faltaron la suma, la resta y la division como operadores aritmeticos.</t>
         </is>
@@ -1550,7 +1546,7 @@
           <t>8</t>
         </is>
       </c>
-      <c r="G34" s="4" t="inlineStr">
+      <c r="G34" s="3" t="inlineStr">
         <is>
           <t>Tu P03 sigue sin estar en tu carpeta: ver tu hoja. T01: 8. Tus operadores estan completos, pero tus atributos no estan etiquetados, no escribiste las firmas, tu main no separa estado inicial, invocaciones y estado final, y Raqueta no tiene un metodo void con parametro. Ademas la subiste a una rama suelta: ver tu hoja.</t>
         </is>
@@ -1587,54 +1583,51 @@
           <t>PC</t>
         </is>
       </c>
-      <c r="G35" s="4" t="inlineStr">
+      <c r="G35" s="3" t="inlineStr">
         <is>
           <t>T01 recibida, pero faltan los tres .class y a los tres comentarios de modelado les falta la linea QUE IGNORE.</t>
         </is>
       </c>
     </row>
-    <row r="36"/>
-    <row r="37"/>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>P00:  calificadas 27   ·   pendientes de correccion 0   ·   sin entregar 2</t>
+          <t>P00:  calificadas 27   ·   pendientes de correccion 0   ·   no entregadas 2</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>P01:  calificadas 26   ·   pendientes de correccion 0   ·   sin entregar 3</t>
+          <t>P01:  calificadas 26   ·   pendientes de correccion 0   ·   no entregadas 3</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>P02:  calificadas 21   ·   pendientes de correccion 2   ·   sin entregar 6</t>
+          <t>P02:  calificadas 21   ·   pendientes de correccion 2   ·   no entregadas 6</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>P03:  calificadas 18   ·   pendientes de correccion 5   ·   sin entregar 6</t>
+          <t>P03:  calificadas 18   ·   pendientes de correccion 5   ·   no entregadas 6</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>T01:  calificadas 9   ·   pendientes de correccion 8   ·   sin entregar 12</t>
-        </is>
-      </c>
-    </row>
-    <row r="43"/>
+          <t>T01:  calificadas 10   ·   pendientes de correccion 8   ·   no entregadas 11</t>
+        </is>
+      </c>
+    </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Cambios desde el 14-sep: se calificaron 3 P03 nuevas y 4 T01 nuevas. Otras 6 T01 llegaron completas pero quedaron pendientes porque les faltan los .class; su codigo compila con JDK 21.</t>
+          <t>Cambios desde el 14-sep: 4 T01 nuevas calificadas, una mas recibida por correo, y 3 P03 nuevas. Seis T01 quedan pendientes solo porque les faltan los .class; su codigo compila con JDK 21.</t>
         </is>
       </c>
     </row>
@@ -1652,8 +1645,8 @@
   <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="62" customWidth="1" style="2" min="1" max="1"/>
-    <col width="72" customWidth="1" style="2" min="2" max="2"/>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1671,51 +1664,50 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>P00: 10    P01: NP    P02: NP    P03: NP    T01: —</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Ya llego tu primera entrega. Faltan la P01, la P02 y la P03.</t>
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Tu P00 quedo en una rama suelta (Shagr33l-patch-1) y no cuenta.</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Copiala a entregas/gutierrez_ixcmie/p00/ en tu rama entregas_gutierrez_ixcmie.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Faltan P01, P02, P03 y T01.</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>Subelas en sus carpetas de tu rama.</t>
         </is>
@@ -1735,8 +1727,8 @@
   <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="62" customWidth="1" style="2" min="1" max="1"/>
-    <col width="72" customWidth="1" style="2" min="2" max="2"/>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1754,63 +1746,62 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>P00: 10    P01: 10    P02: NP    P03: PC    T01: —</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>P03 recibida y con 35 de 36 aciertos, pero falta el documento con las explicaciones y tu carpeta esta escrita 'hermenegilo_eduardo', sin la d. Renombrala a hermenegildo_eduardo.</t>
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Tu carpeta se llama hermenegilo_eduardo, sin la d.</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Renombrala a hermenegildo_eduardo para que quede junto a tu P00 y P01.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Falta el documento con las explicaciones de la P03.</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>Explica por que fallaste cada expresion; acertaste 35 de 36, asi que es corto.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>Falta la T01.</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>3 .java, 3 .class y QUIZ.md en tareas/t01/.</t>
         </is>
@@ -1827,11 +1818,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="62" customWidth="1" style="2" min="1" max="1"/>
-    <col width="72" customWidth="1" style="2" min="2" max="2"/>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1849,41 +1840,76 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t>P00: 10    P01: 9    P02: 10    P03: 10    T01: —</t>
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>P00: 10    P01: 9    P02: 10    P03: 10    T01: 8</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
-        <is>
-          <t>Tu P03 esta completa y bien explicada. Detalle: en tu comentario del 7.2 escribiste 'primo' donde querias decir 'par'.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5"/>
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>T01 entregada por correo, no por Git: dice que creo las ramas pero no lo dejo hacer push. Los .class corren con JDK 21 y el quiz trae las 10 respuestas con tus palabras. Le falta el comentario de modelado en las cuatro lineas etiquetadas, el '// firma:' de cada metodo y que cada objeto tenga su propio main; por eso 8. Falta subirla a entregas/hernandez_mauricio/tareas/t01/.</t>
+        </is>
+      </c>
+    </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
-        <is>
-          <t>Falta la T01.</t>
-        </is>
-      </c>
-      <c r="B7" s="4" t="inlineStr">
-        <is>
-          <t>Tu rama t01-HernandezGonzalez solo tiene practicas viejas. Sube la tarea en entregas/hernandez_mauricio/tareas/t01/, en tu rama entregas_hernandez_mauricio.</t>
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Tu T01 llego por correo y no esta en el repo.</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Subela a entregas/hernandez_mauricio/tareas/t01/ en tu rama entregas_hernandez_mauricio. Si el push sigue fallando, escribeme y lo vemos en un zoom.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Tus comentarios de modelado son prosa corrida.</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Van en cuatro lineas etiquetadas: CONTEXTO, QUE SABE Y POR QUE, QUE SABE HACER Y POR QUE, QUE IGNORE.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Ningun metodo trae su firma en comentario.</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Agrega // firma: metodo(tipo) arriba de cada uno.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Celular no tiene su propio main y dos objetos piden datos por teclado.</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>El enunciado pide que cada objeto tenga su main con estado inicial, invocaciones y estado final, sin Scanner.</t>
         </is>
       </c>
     </row>
@@ -1901,8 +1927,8 @@
   <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="62" customWidth="1" style="2" min="1" max="1"/>
-    <col width="72" customWidth="1" style="2" min="2" max="2"/>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1920,51 +1946,50 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>P00: 10    P01: 10    P02: 10    P03: 10    T01: 9</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>T01 completa y corriendo. Detalles: los tres programas imprimen 'RADIOGRAFIA: MiObjeto', que es el titulo de la plantilla, y a dos comentarios les falta la linea QUE IGNORE.</t>
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Los tres programas imprimen 'RADIOGRAFIA: MiObjeto'.</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Cambia ese titulo por el nombre real de cada clase.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>A dos comentarios les falta la linea QUE IGNORE.</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>Agregala: una o dos cosas del objeto real que no modelaste, y por que.</t>
         </is>
@@ -1984,8 +2009,8 @@
   <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="62" customWidth="1" style="2" min="1" max="1"/>
-    <col width="72" customWidth="1" style="2" min="2" max="2"/>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2003,39 +2028,38 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>P00: 10    P01: 10    P02: 9    P03: 10    T01: 9</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>T01 completa y corriendo. Un detalle: la subiste a entregas/hernandez_emily/t01/ y va en entregas/hernandez_emily/tareas/t01/.</t>
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Tu T01 esta en entregas/hernandez_emily/t01/.</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Muevela a entregas/hernandez_emily/tareas/t01/, que es la ruta del enunciado.</t>
         </is>
@@ -2055,8 +2079,8 @@
   <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="62" customWidth="1" style="2" min="1" max="1"/>
-    <col width="72" customWidth="1" style="2" min="2" max="2"/>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2074,39 +2098,38 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>P00: 10    P01: 9    P02: 9    P03: 10    T01: PC</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>El mejor analisis del grupo, aceptada. Para que lo tengas: tu 7.2 imprime true y se pedia false, y tu documento no trae tu nombre. T01: le falta casi todo lo que se califica: comentario de modelado, etiquetas, firmas, los .class, tipos y varios operadores. Ver tu hoja.</t>
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Sigue pendiente lo del 14-sep.</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Revisa la observacion de tu corte anterior y sube el arreglo; avisame cuando este.</t>
         </is>
@@ -2126,8 +2149,8 @@
   <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="62" customWidth="1" style="2" min="1" max="1"/>
-    <col width="72" customWidth="1" style="2" min="2" max="2"/>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2145,75 +2168,74 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>P00: 10    P01: 10    P02: 9    P03: 9    T01: PC</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>T01 recibida, pero faltan los tres .class, el quiz debe llamarse QUIZ.md (subiste 'Quiz de la T01.txt'), la carpeta va en minusculas (tareas/t01) y ningun metodo trae su '// firma:'.</t>
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Tu T01 no trae los .class.</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Compila los tres con JDK 21 y subelos.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>El quiz se llama 'Quiz de la T01.txt'.</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>Debe ser QUIZ.md.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>Tu carpeta es Tareas/T01, con mayusculas.</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>Usa tareas/t01 en minusculas.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>Ningun metodo trae su firma en comentario.</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>Agrega // firma: metodo(tipo) arriba de cada metodo.</t>
         </is>
@@ -2233,8 +2255,8 @@
   <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="62" customWidth="1" style="2" min="1" max="1"/>
-    <col width="72" customWidth="1" style="2" min="2" max="2"/>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2252,51 +2274,50 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>P00: 10    P01: 10    P02: PC    P03: 8    T01: —</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Aceptada tu P03 en 8 (ver tu hoja). Llegaron tu P01, que esta bien, y tu P02, que no compila: tambien en tu hoja.</t>
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Tu P02 sigue pendiente desde el 14-sep.</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Revisa la observacion anterior y sube el arreglo.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Falta la T01.</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>3 .java, 3 .class y QUIZ.md en tareas/t01/.</t>
         </is>
@@ -2316,8 +2337,8 @@
   <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="62" customWidth="1" style="2" min="1" max="1"/>
-    <col width="72" customWidth="1" style="2" min="2" max="2"/>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2335,39 +2356,38 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>P00: 10    P01: 10    P02: 10    P03: 9    T01: —</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Tu bloque 7 esta completo y eres el unico que puso el comentario del operador en cada linea. Falto la captura de la TABLA FINAL, que era lo que se pedia, y tu analisis va por temas en vez de falla por falla.</t>
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Falta la T01.</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>3 .java, 3 .class y QUIZ.md en entregas/medina_miguel/tareas/t01/.</t>
         </is>
@@ -2387,8 +2407,8 @@
   <dimension ref="A1:B9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="62" customWidth="1" style="2" min="1" max="1"/>
-    <col width="72" customWidth="1" style="2" min="2" max="2"/>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2406,63 +2426,62 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>P00: 10    P01: 9    P02: 10    P03: 10    T01: —</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>P03 lista: tabla completa y el mejor analisis del grupo, con tus palabras. Dos cosas de orden: tu carpeta se llama diego_mendez y deberia ser mendez_juan, donde estan tu P00 y P01, y tienes dos ramas de entregas; trabaja solo en entregas_mendez_juan.</t>
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Tu carpeta se llama diego_mendez.</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Deberia ser mendez_juan, donde estan tu P00 y tu P01.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Tienes dos ramas de entregas.</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>Trabaja solo en entregas_mendez_juan; la otra ya no la uses.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>Falta la T01.</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>3 .java, 3 .class y QUIZ.md en tareas/t01/.</t>
         </is>
@@ -2482,8 +2501,8 @@
   <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="62" customWidth="1" style="2" min="1" max="1"/>
-    <col width="72" customWidth="1" style="2" min="2" max="2"/>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2501,39 +2520,38 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>P00: 10    P01: 9    P02: 10    P03: 10    T01: —</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>P03 lista: tabla completa y analisis en el PDF (documento conjunto con otros dos companeros). En mis-resultados.txt dejaste en blanco los 'por que me equivoque', pero estan explicados en el PDF. Falta la T01.</t>
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Falta la T01 completa.</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Sube los 3 .java, sus 3 .class y QUIZ.md en entregas/ajas_andre/tareas/t01/.</t>
         </is>
@@ -2553,8 +2571,8 @@
   <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="62" customWidth="1" style="2" min="1" max="1"/>
-    <col width="72" customWidth="1" style="2" min="2" max="2"/>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2572,39 +2590,38 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>P00: NP    P01: NP    P02: NP    P03: NP    T01: —</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Sin entregas registradas.</t>
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>No hay ninguna entrega tuya en el repo.</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Crea tu rama entregas_olmedo_marco y sube P00, P01, P02 y P03; despues la T01.</t>
         </is>
@@ -2624,8 +2641,8 @@
   <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="62" customWidth="1" style="2" min="1" max="1"/>
-    <col width="72" customWidth="1" style="2" min="2" max="2"/>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2643,51 +2660,50 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>P00: 10    P01: 9    P02: 10    P03: PC    T01: PC</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Sigue igual que el 14-sep: tu T01 esta completa (compila y el quiz tiene las 10 respuestas) pero vive en entregas/Paula_Romero/, suelta y sin .class. Muevela a entregas/romero_paula/tareas/t01/, agrega los .class y mueve tambien la P03.</t>
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Tu T01 esta completa pero suelta en entregas/Paula_Romero/.</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Muevela a entregas/romero_paula/tareas/t01/ y agrega los tres .class; tu codigo ya compila con JDK 21.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Tu P03 tambien esta en esa carpeta.</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>Muevela a entregas/romero_paula/p03/.</t>
         </is>
@@ -2707,8 +2723,8 @@
   <dimension ref="A1:B10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="62" customWidth="1" style="2" min="1" max="1"/>
-    <col width="72" customWidth="1" style="2" min="2" max="2"/>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2726,75 +2742,74 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>P00: 10    P01: 9    P02: 10    P03: PC    T01: PC</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>T01 recibida, pero faltan los tres .class, el quiz solo trae 2 de las 10 respuestas y subiste MiObjeto.java, que es la plantilla sin llenar.</t>
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Tu T01 no trae los .class.</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Compila los tres con JDK 21 y subelos.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>El quiz solo tiene 2 de las 10 respuestas.</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>Completa las otras ocho, con tus palabras.</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="4" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t>Subiste MiObjeto.java, que es la plantilla sin llenar.</t>
         </is>
       </c>
-      <c r="B9" s="4" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t>Borrala de tu carpeta.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="4" t="inlineStr">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>Tu P03 sigue pendiente desde el 14-sep.</t>
         </is>
       </c>
-      <c r="B10" s="4" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>Revisa la observacion anterior y sube el arreglo.</t>
         </is>
@@ -2814,8 +2829,8 @@
   <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="62" customWidth="1" style="2" min="1" max="1"/>
-    <col width="72" customWidth="1" style="2" min="2" max="2"/>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2833,39 +2848,38 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>P00: 10    P01: 10    P02: 10    P03: PC    T01: 9</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Incompleta: en tu carpeta solo esta el Laboratorio.class. Aunque el trabajo sea de equipo, cada quien sube su .java y su documento con la captura y el analisis. Ver tu hoja. T01: 9, pero esta en una rama suelta: pasala a tu rama del semestre (ver tu hoja). Entre tus clases faltaron la suma, la resta y la division como operadores aritmeticos.</t>
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>En tu p03 solo esta Laboratorio.class.</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Sube tambien Laboratorio.java y mis-resultados.txt con tu tabla.</t>
         </is>
@@ -2885,8 +2899,8 @@
   <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="62" customWidth="1" style="2" min="1" max="1"/>
-    <col width="72" customWidth="1" style="2" min="2" max="2"/>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2904,39 +2918,38 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>P00: 10    P01: 10    P02: 10    P03: PC    T01: 8</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Tu P03 sigue sin estar en tu carpeta: ver tu hoja. T01: 8. Tus operadores estan completos, pero tus atributos no estan etiquetados, no escribiste las firmas, tu main no separa estado inicial, invocaciones y estado final, y Raqueta no tiene un metodo void con parametro. Ademas la subiste a una rama suelta: ver tu hoja.</t>
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Tu P03 sigue pendiente desde el 14-sep.</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Revisa la observacion anterior y sube el arreglo.</t>
         </is>
@@ -2956,8 +2969,8 @@
   <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="62" customWidth="1" style="2" min="1" max="1"/>
-    <col width="72" customWidth="1" style="2" min="2" max="2"/>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -2975,51 +2988,50 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>P00: 10    P01: 10    P02: 10    P03: 9    T01: PC</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>T01 recibida, pero faltan los tres .class y a los tres comentarios de modelado les falta la linea QUE IGNORE.</t>
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Tu T01 no trae los .class.</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Compila los tres con JDK 21 y subelos.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>A los tres comentarios les falta la linea QUE IGNORE.</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>Agregala en cada clase.</t>
         </is>
@@ -3039,8 +3051,8 @@
   <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="62" customWidth="1" style="2" min="1" max="1"/>
-    <col width="72" customWidth="1" style="2" min="2" max="2"/>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3058,39 +3070,38 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>P00: 10    P01: 10    P02: 10    P03: 10    T01: PC</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Tu T01 quedo sin los .class: los borraste el 21-sep. El codigo compila bien con JDK 21 y el modelado y el quiz estan muy completos; recompila los tres y subelos para cerrarla.</t>
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Borraste tus tres .class el 21-sep, y la T01 se califica ejecutandolos.</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Compila con el JDK 21 (javac Bicicleta.java, etc.), pruebalo con java Bicicleta y sube los tres .class junto a tus .java.</t>
         </is>
@@ -3110,8 +3121,8 @@
   <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="62" customWidth="1" style="2" min="1" max="1"/>
-    <col width="72" customWidth="1" style="2" min="2" max="2"/>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3129,51 +3140,50 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>P00: 10    P01: 10    P02: NP    P03: NP    T01: —</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Faltan la P02 y la P03.</t>
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>No tienes P02 ni P03.</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Sube la P02 en entregas/castillo_ihsahn/p02/ y la P03 en p03/, con Laboratorio.java y mis-resultados.txt.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Falta la T01.</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>3 .java, 3 .class y QUIZ.md en tareas/t01/.</t>
         </is>
@@ -3193,8 +3203,8 @@
   <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="62" customWidth="1" style="2" min="1" max="1"/>
-    <col width="72" customWidth="1" style="2" min="2" max="2"/>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3212,51 +3222,50 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>P00: 10    P01: 10    P02: 10    P03: 10    T01: PC</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>P03 lista: tabla de 41 filas con analisis en PDF y captura. En la T01 faltan los tres .class y ningun metodo trae su '// firma:' en comentario.</t>
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Tu T01 no trae los .class.</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Compila los tres con JDK 21 y subelos.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Ningun metodo trae su firma en comentario.</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>Agrega // firma: metodo(tipo) arriba de cada metodo, como pide el enunciado.</t>
         </is>
@@ -3276,8 +3285,8 @@
   <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="62" customWidth="1" style="2" min="1" max="1"/>
-    <col width="72" customWidth="1" style="2" min="2" max="2"/>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3295,39 +3304,38 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>P00: NP    P01: NP    P02: NP    P03: NP    T01: —</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Sin entregas registradas.</t>
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>No hay ninguna entrega tuya en el repo.</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Crea tu rama entregas_cruz_isaac y sube P00, P01, P02 y P03; despues la T01.</t>
         </is>
@@ -3347,8 +3355,8 @@
   <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="62" customWidth="1" style="2" min="1" max="1"/>
-    <col width="72" customWidth="1" style="2" min="2" max="2"/>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3366,51 +3374,50 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>P00: 10    P01: 10    P02: 10    P03: 10    T01: PC</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>T01 recibida, pero faltan los tres .class y dejaste dentro de los comentarios y del quiz las preguntas de la plantilla (los parentesis con instrucciones). Borralos y sube los .class.</t>
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Tu T01 no trae los .class.</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Compila los tres con JDK 21 y subelos.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>Dejaste las preguntas de la plantilla dentro de los comentarios y del quiz.</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>Borra los parentesis con las instrucciones y deja solo tu respuesta.</t>
         </is>
@@ -3430,8 +3437,8 @@
   <dimension ref="A1:B8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="62" customWidth="1" style="2" min="1" max="1"/>
-    <col width="72" customWidth="1" style="2" min="2" max="2"/>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3449,51 +3456,50 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>P00: 10    P01: 10    P02: PC    P03: NP    T01: —</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Tu P02 sigue sin compilar. Falta la P03. Ver tu hoja.</t>
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>Tu P02 no compila.</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Arregla PruebaPunto para que corra y vuelve a subirla.</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="4" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t>No tienes P03 ni T01.</t>
         </is>
       </c>
-      <c r="B8" s="4" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t>Sube la P03 en p03/ y la T01 en tareas/t01/.</t>
         </is>
@@ -3513,8 +3519,8 @@
   <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="62" customWidth="1" style="2" min="1" max="1"/>
-    <col width="72" customWidth="1" style="2" min="2" max="2"/>
+    <col width="62" customWidth="1" min="1" max="1"/>
+    <col width="72" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -3532,39 +3538,38 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="4" t="inlineStr">
         <is>
           <t>P00: 10    P01: 9    P02: NP    P03: NP    T01: —</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="4" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t>Tu HolaMundo no lleva tu nombre. Faltan la P02 y la P03.</t>
         </is>
       </c>
     </row>
-    <row r="5"/>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Que hay que corregir</t>
         </is>
       </c>
-      <c r="B6" s="3" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>Como se corrige</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="4" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t>No tienes P02, P03 ni T01.</t>
         </is>
       </c>
-      <c r="B7" s="4" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t>Sube cada una en su carpeta dentro de entregas/gonzalez_ramon/.</t>
         </is>

</xml_diff>